<commit_message>
UK daily ratings for 2026-05-31
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-31.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-31.xlsx
@@ -526,14 +526,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Ocean Club (IRE)</t>
+          <t>High Morals (USA)</t>
         </is>
       </c>
       <c r="I2" t="n">
         <v>2</v>
       </c>
       <c r="J2" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -580,7 +580,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>No Time Faults (IRE)</t>
+          <t>Scarlet Dream (IRE)</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -634,14 +634,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>High Morals (USA)</t>
+          <t>Portaliffe Phil (IRE)</t>
         </is>
       </c>
       <c r="I4" t="n">
         <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -688,14 +688,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Scarlet Dream (IRE)</t>
+          <t>Ocean Club (IRE)</t>
         </is>
       </c>
       <c r="I5" t="n">
         <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -742,14 +742,14 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Portaliffe Phil (IRE)</t>
+          <t>No Time Faults (IRE)</t>
         </is>
       </c>
       <c r="I6" t="n">
         <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -1894,17 +1894,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Amicitia (IRE)</t>
+          <t>Famed Again (IRE)</t>
         </is>
       </c>
       <c r="I26" t="n">
         <v>4</v>
       </c>
       <c r="J26" t="n">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="K26" t="n">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -1948,17 +1948,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Famed Again (IRE)</t>
+          <t>Little Empire (IRE)</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J27" t="n">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="K27" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2002,17 +2002,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Little Empire (IRE)</t>
+          <t>Amicitia (IRE)</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="K28" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -3258,17 +3258,17 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Sovereign Banter (IRE)</t>
+          <t>Rockbury Lad</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J50" t="n">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="K50" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="n">
@@ -3312,17 +3312,17 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Rockbury Lad</t>
+          <t>Sovereign Banter (IRE)</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J51" t="n">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="K51" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="n">
@@ -4234,17 +4234,17 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Loyal Touch (IRE)</t>
+          <t>Parish Express (IRE)</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J67" t="n">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="K67" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="n">
@@ -4288,17 +4288,17 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Parish Express (IRE)</t>
+          <t>Tassarolo</t>
         </is>
       </c>
       <c r="I68" t="n">
         <v>5</v>
       </c>
       <c r="J68" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K68" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="n">
@@ -4342,17 +4342,17 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Tassarolo</t>
+          <t>Loyal Touch (IRE)</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J69" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="K69" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="n">

</xml_diff>